<commit_message>
Update scripts and data files: 35_프로젝트계획서최신화이력관리
</commit_message>
<xml_diff>
--- a/data/자동화태스크.xlsx
+++ b/data/자동화태스크.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWork\MySite\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWork\MySite\stComm\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="299">
   <si>
     <r>
       <rPr>
@@ -72922,6 +72922,2204 @@
       </rPr>
       <t>_MSTeams.html</t>
     </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>IHANS_PRO_2026_035</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트계획서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>및</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>업데이트</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>착수시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>및</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마일스톤마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>여부를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>리뷰하고나서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>필요시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>업데이트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>초기에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성된</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>끝날</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>때까지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> v1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>유지되는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>경우가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>많다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>심사를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>대비한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사문서로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>여기지고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>심사에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>많은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>지적이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>발생하는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>것이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>현실이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마일스톤</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>여부를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>점검하기로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>규정한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>다만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마일스톤마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>반드시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>되어야</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>하는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>것은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>아니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>될</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>때마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>버전이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>하나씩</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>올라간다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종료될</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>때까지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> v1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>유지하더라도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>마일스톤마다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>여부를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>점검하였다는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기록이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>남는다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>과정에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>포함되지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>않는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>항목이</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>과정에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>생성될</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>있으며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트계획서가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>살아있는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>문서임을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>증빙하는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사례가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>된다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최신화되는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>경우에도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기존</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>내용은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>유지하도록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>하여</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>변경</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>내용을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>확인할</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>있도록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>35_프로젝트계획서최신화이력관리.html</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -73322,33 +75520,6 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -73396,6 +75567,33 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -73796,10 +75994,10 @@
       <c r="G3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="29" t="s">
+      <c r="H3" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="I3" s="29"/>
+      <c r="I3" s="45"/>
     </row>
     <row r="4" spans="2:11" s="11" customFormat="1" ht="26">
       <c r="B4" s="6" t="s">
@@ -73832,7 +76030,7 @@
       <c r="B5" s="12">
         <v>1</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="46" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="13" t="s">
@@ -73844,7 +76042,7 @@
       <c r="F5" s="14">
         <v>90</v>
       </c>
-      <c r="G5" s="31" t="s">
+      <c r="G5" s="47" t="s">
         <v>14</v>
       </c>
       <c r="H5" s="15" t="s">
@@ -73860,7 +76058,7 @@
       <c r="B6" s="12">
         <v>2</v>
       </c>
-      <c r="C6" s="30"/>
+      <c r="C6" s="46"/>
       <c r="D6" s="13" t="s">
         <v>17</v>
       </c>
@@ -73870,7 +76068,7 @@
       <c r="F6" s="14">
         <v>90</v>
       </c>
-      <c r="G6" s="31"/>
+      <c r="G6" s="47"/>
       <c r="H6" s="15" t="s">
         <v>19</v>
       </c>
@@ -73883,7 +76081,7 @@
       <c r="B7" s="12">
         <v>3</v>
       </c>
-      <c r="C7" s="30"/>
+      <c r="C7" s="46"/>
       <c r="D7" s="13" t="s">
         <v>21</v>
       </c>
@@ -73906,7 +76104,7 @@
       <c r="B8" s="12">
         <v>4</v>
       </c>
-      <c r="C8" s="30"/>
+      <c r="C8" s="46"/>
       <c r="D8" s="13" t="s">
         <v>25</v>
       </c>
@@ -73927,7 +76125,7 @@
       <c r="B9" s="12">
         <v>5</v>
       </c>
-      <c r="C9" s="30"/>
+      <c r="C9" s="46"/>
       <c r="D9" s="13" t="s">
         <v>28</v>
       </c>
@@ -73953,7 +76151,7 @@
       <c r="B10" s="12">
         <v>6</v>
       </c>
-      <c r="C10" s="30"/>
+      <c r="C10" s="46"/>
       <c r="D10" s="13" t="s">
         <v>33</v>
       </c>
@@ -73978,7 +76176,7 @@
       <c r="B11" s="12">
         <v>7</v>
       </c>
-      <c r="C11" s="30"/>
+      <c r="C11" s="46"/>
       <c r="D11" s="13" t="s">
         <v>38</v>
       </c>
@@ -74003,7 +76201,7 @@
       <c r="B12" s="12">
         <v>8</v>
       </c>
-      <c r="C12" s="30"/>
+      <c r="C12" s="46"/>
       <c r="D12" s="13" t="s">
         <v>43</v>
       </c>
@@ -74028,7 +76226,7 @@
       <c r="B13" s="12">
         <v>9</v>
       </c>
-      <c r="C13" s="30"/>
+      <c r="C13" s="46"/>
       <c r="D13" s="13" t="s">
         <v>48</v>
       </c>
@@ -74053,7 +76251,7 @@
       <c r="B14" s="12">
         <v>10</v>
       </c>
-      <c r="C14" s="30"/>
+      <c r="C14" s="46"/>
       <c r="D14" s="13" t="s">
         <v>53</v>
       </c>
@@ -74078,7 +76276,7 @@
       <c r="B15" s="12">
         <v>11</v>
       </c>
-      <c r="C15" s="30"/>
+      <c r="C15" s="46"/>
       <c r="D15" s="13" t="s">
         <v>58</v>
       </c>
@@ -74099,7 +76297,7 @@
       <c r="B16" s="12">
         <v>12</v>
       </c>
-      <c r="C16" s="30"/>
+      <c r="C16" s="46"/>
       <c r="D16" s="13" t="s">
         <v>61</v>
       </c>
@@ -74124,7 +76322,7 @@
       <c r="B17" s="12">
         <v>13</v>
       </c>
-      <c r="C17" s="30"/>
+      <c r="C17" s="46"/>
       <c r="D17" s="13" t="s">
         <v>66</v>
       </c>
@@ -74147,7 +76345,7 @@
       <c r="B18" s="12">
         <v>14</v>
       </c>
-      <c r="C18" s="32" t="s">
+      <c r="C18" s="48" t="s">
         <v>70</v>
       </c>
       <c r="D18" s="15" t="s">
@@ -74172,7 +76370,7 @@
       <c r="B19" s="12">
         <v>15</v>
       </c>
-      <c r="C19" s="33"/>
+      <c r="C19" s="49"/>
       <c r="D19" s="13" t="s">
         <v>75</v>
       </c>
@@ -74195,7 +76393,7 @@
       <c r="B20" s="12">
         <v>16</v>
       </c>
-      <c r="C20" s="33"/>
+      <c r="C20" s="49"/>
       <c r="D20" s="13" t="s">
         <v>79</v>
       </c>
@@ -74218,7 +76416,7 @@
       <c r="B21" s="12">
         <v>17</v>
       </c>
-      <c r="C21" s="33"/>
+      <c r="C21" s="49"/>
       <c r="D21" s="13" t="s">
         <v>82</v>
       </c>
@@ -74241,7 +76439,7 @@
       <c r="B22" s="12">
         <v>18</v>
       </c>
-      <c r="C22" s="33"/>
+      <c r="C22" s="49"/>
       <c r="D22" s="13" t="s">
         <v>86</v>
       </c>
@@ -74266,7 +76464,7 @@
       <c r="B23" s="12">
         <v>19</v>
       </c>
-      <c r="C23" s="33"/>
+      <c r="C23" s="49"/>
       <c r="D23" s="13" t="s">
         <v>90</v>
       </c>
@@ -74289,7 +76487,7 @@
       <c r="B24" s="12">
         <v>20</v>
       </c>
-      <c r="C24" s="33"/>
+      <c r="C24" s="49"/>
       <c r="D24" s="13" t="s">
         <v>94</v>
       </c>
@@ -74312,7 +76510,7 @@
       <c r="B25" s="12">
         <v>21</v>
       </c>
-      <c r="C25" s="33"/>
+      <c r="C25" s="49"/>
       <c r="D25" s="13" t="s">
         <v>98</v>
       </c>
@@ -74337,7 +76535,7 @@
       <c r="B26" s="12">
         <v>22</v>
       </c>
-      <c r="C26" s="33"/>
+      <c r="C26" s="49"/>
       <c r="D26" s="13" t="s">
         <v>103</v>
       </c>
@@ -74362,7 +76560,7 @@
       <c r="B27" s="12">
         <v>23</v>
       </c>
-      <c r="C27" s="33"/>
+      <c r="C27" s="49"/>
       <c r="D27" s="13" t="s">
         <v>108</v>
       </c>
@@ -74385,7 +76583,7 @@
       <c r="B28" s="12">
         <v>24</v>
       </c>
-      <c r="C28" s="33"/>
+      <c r="C28" s="49"/>
       <c r="D28" s="13" t="s">
         <v>112</v>
       </c>
@@ -74410,7 +76608,7 @@
       <c r="B29" s="12">
         <v>25</v>
       </c>
-      <c r="C29" s="34"/>
+      <c r="C29" s="50"/>
       <c r="D29" s="13" t="s">
         <v>117</v>
       </c>
@@ -74435,7 +76633,7 @@
       <c r="B30" s="12">
         <v>26</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="46" t="s">
         <v>122</v>
       </c>
       <c r="D30" s="13" t="s">
@@ -74458,7 +76656,7 @@
       <c r="B31" s="12">
         <v>27</v>
       </c>
-      <c r="C31" s="30"/>
+      <c r="C31" s="46"/>
       <c r="D31" s="13" t="s">
         <v>127</v>
       </c>
@@ -74483,7 +76681,7 @@
       <c r="B32" s="12">
         <v>28</v>
       </c>
-      <c r="C32" s="30"/>
+      <c r="C32" s="46"/>
       <c r="D32" s="13" t="s">
         <v>131</v>
       </c>
@@ -74506,7 +76704,7 @@
       <c r="B33" s="12">
         <v>29</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="46" t="s">
         <v>135</v>
       </c>
       <c r="D33" s="13" t="s">
@@ -74533,7 +76731,7 @@
       <c r="B34" s="12">
         <v>30</v>
       </c>
-      <c r="C34" s="30"/>
+      <c r="C34" s="46"/>
       <c r="D34" s="13" t="s">
         <v>140</v>
       </c>
@@ -74556,7 +76754,7 @@
       <c r="B35" s="12">
         <v>31</v>
       </c>
-      <c r="C35" s="32"/>
+      <c r="C35" s="48"/>
       <c r="D35" s="13" t="s">
         <v>144</v>
       </c>
@@ -74581,7 +76779,7 @@
       <c r="B36" s="12">
         <v>32</v>
       </c>
-      <c r="C36" s="26" t="s">
+      <c r="C36" s="42" t="s">
         <v>148</v>
       </c>
       <c r="D36" s="21" t="s">
@@ -74605,7 +76803,7 @@
       <c r="B37" s="12">
         <v>33</v>
       </c>
-      <c r="C37" s="27"/>
+      <c r="C37" s="43"/>
       <c r="D37" s="21" t="s">
         <v>153</v>
       </c>
@@ -74627,7 +76825,7 @@
       <c r="B38" s="12">
         <v>34</v>
       </c>
-      <c r="C38" s="28"/>
+      <c r="C38" s="44"/>
       <c r="D38" s="21" t="s">
         <v>157</v>
       </c>
@@ -74667,7 +76865,7 @@
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K38"/>
+  <dimension ref="B2:K39"/>
   <sheetFormatPr defaultRowHeight="11.5"/>
   <cols>
     <col min="1" max="1" width="2.58203125" style="2" customWidth="1"/>
@@ -74688,42 +76886,42 @@
       </c>
     </row>
     <row r="3" spans="2:11" ht="17" customHeight="1">
-      <c r="B3" s="48"/>
-      <c r="C3" s="49"/>
-      <c r="D3" s="50"/>
-      <c r="E3" s="49"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="50"/>
-      <c r="H3" s="50"/>
+      <c r="B3" s="39"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="2:11" s="11" customFormat="1" ht="13">
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="29" t="s">
         <v>197</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="30" t="s">
         <v>196</v>
       </c>
-      <c r="E4" s="40" t="s">
+      <c r="E4" s="31" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="41" t="s">
+      <c r="F4" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="42" t="s">
+      <c r="G4" s="33" t="s">
         <v>212</v>
       </c>
-      <c r="H4" s="43" t="s">
+      <c r="H4" s="34" t="s">
         <v>247</v>
       </c>
-      <c r="K4" s="47" t="s">
+      <c r="K4" s="38" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="5" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B5" s="44">
+      <c r="B5" s="35">
         <v>1</v>
       </c>
       <c r="C5" s="25" t="s">
@@ -74735,20 +76933,20 @@
       <c r="E5" s="25" t="s">
         <v>198</v>
       </c>
-      <c r="F5" s="45"/>
-      <c r="G5" s="46" t="s">
+      <c r="F5" s="36"/>
+      <c r="G5" s="37" t="s">
         <v>252</v>
       </c>
-      <c r="H5" s="45" t="s">
+      <c r="H5" s="36" t="s">
         <v>213</v>
       </c>
       <c r="I5" s="17"/>
-      <c r="K5" s="47" t="s">
+      <c r="K5" s="38" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="6" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B6" s="44">
+      <c r="B6" s="35">
         <v>2</v>
       </c>
       <c r="C6" s="25" t="s">
@@ -74760,21 +76958,21 @@
       <c r="E6" s="25" t="s">
         <v>199</v>
       </c>
-      <c r="F6" s="45" t="s">
+      <c r="F6" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="45" t="s">
+      <c r="G6" s="36" t="s">
         <v>261</v>
       </c>
-      <c r="H6" s="45" t="s">
+      <c r="H6" s="36" t="s">
         <v>214</v>
       </c>
-      <c r="K6" s="47" t="s">
+      <c r="K6" s="38" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="7" spans="2:11" s="11" customFormat="1" ht="182.5" customHeight="1">
-      <c r="B7" s="44">
+      <c r="B7" s="35">
         <v>3</v>
       </c>
       <c r="C7" s="25" t="s">
@@ -74786,21 +76984,21 @@
       <c r="E7" s="25" t="s">
         <v>200</v>
       </c>
-      <c r="F7" s="45" t="s">
+      <c r="F7" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="36" t="s">
         <v>262</v>
       </c>
-      <c r="H7" s="45" t="s">
+      <c r="H7" s="36" t="s">
         <v>215</v>
       </c>
-      <c r="K7" s="47" t="s">
+      <c r="K7" s="38" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="8" spans="2:11" s="11" customFormat="1" ht="182.5" customHeight="1">
-      <c r="B8" s="44">
+      <c r="B8" s="35">
         <v>4</v>
       </c>
       <c r="C8" s="25" t="s">
@@ -74812,19 +77010,19 @@
       <c r="E8" s="25" t="s">
         <v>248</v>
       </c>
-      <c r="F8" s="45"/>
-      <c r="G8" s="45" t="s">
+      <c r="F8" s="36"/>
+      <c r="G8" s="36" t="s">
         <v>253</v>
       </c>
-      <c r="H8" s="45" t="s">
+      <c r="H8" s="36" t="s">
         <v>216</v>
       </c>
-      <c r="K8" s="47" t="s">
+      <c r="K8" s="38" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="9" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B9" s="44">
+      <c r="B9" s="35">
         <v>5</v>
       </c>
       <c r="C9" s="25" t="s">
@@ -74836,19 +77034,19 @@
       <c r="E9" s="25" t="s">
         <v>249</v>
       </c>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45" t="s">
+      <c r="F9" s="36"/>
+      <c r="G9" s="36" t="s">
         <v>254</v>
       </c>
-      <c r="H9" s="45" t="s">
+      <c r="H9" s="36" t="s">
         <v>217</v>
       </c>
-      <c r="K9" s="47" t="s">
+      <c r="K9" s="38" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="10" spans="2:11" s="11" customFormat="1" ht="26">
-      <c r="B10" s="44">
+      <c r="B10" s="35">
         <v>6</v>
       </c>
       <c r="C10" s="25" t="s">
@@ -74860,40 +77058,40 @@
       <c r="E10" s="25" t="s">
         <v>201</v>
       </c>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45" t="s">
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36" t="s">
         <v>218</v>
       </c>
-      <c r="K10" s="47" t="s">
+      <c r="K10" s="38" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="11" spans="2:11" s="11" customFormat="1" ht="104">
-      <c r="B11" s="44">
+      <c r="B11" s="35">
         <v>7</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>188</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="36" t="s">
         <v>176</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>250</v>
       </c>
-      <c r="F11" s="45"/>
-      <c r="G11" s="45" t="s">
+      <c r="F11" s="36"/>
+      <c r="G11" s="36" t="s">
         <v>255</v>
       </c>
-      <c r="H11" s="45" t="s">
+      <c r="H11" s="36" t="s">
         <v>219</v>
       </c>
       <c r="I11" s="17"/>
-      <c r="K11" s="35"/>
+      <c r="K11" s="26"/>
     </row>
     <row r="12" spans="2:11" s="11" customFormat="1" ht="78">
-      <c r="B12" s="44">
+      <c r="B12" s="35">
         <v>8</v>
       </c>
       <c r="C12" s="25" t="s">
@@ -74905,17 +77103,17 @@
       <c r="E12" s="25" t="s">
         <v>251</v>
       </c>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45" t="s">
+      <c r="F12" s="36"/>
+      <c r="G12" s="36" t="s">
         <v>256</v>
       </c>
-      <c r="H12" s="45" t="s">
+      <c r="H12" s="36" t="s">
         <v>220</v>
       </c>
-      <c r="K12" s="35"/>
+      <c r="K12" s="26"/>
     </row>
     <row r="13" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B13" s="44">
+      <c r="B13" s="35">
         <v>9</v>
       </c>
       <c r="C13" s="25" t="s">
@@ -74927,17 +77125,17 @@
       <c r="E13" s="25" t="s">
         <v>202</v>
       </c>
-      <c r="F13" s="45"/>
-      <c r="G13" s="45" t="s">
+      <c r="F13" s="36"/>
+      <c r="G13" s="36" t="s">
         <v>257</v>
       </c>
-      <c r="H13" s="45" t="s">
+      <c r="H13" s="36" t="s">
         <v>221</v>
       </c>
-      <c r="K13" s="35"/>
+      <c r="K13" s="26"/>
     </row>
     <row r="14" spans="2:11" s="11" customFormat="1" ht="78">
-      <c r="B14" s="44">
+      <c r="B14" s="35">
         <v>10</v>
       </c>
       <c r="C14" s="25" t="s">
@@ -74949,17 +77147,17 @@
       <c r="E14" s="25" t="s">
         <v>203</v>
       </c>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45" t="s">
+      <c r="F14" s="36"/>
+      <c r="G14" s="36" t="s">
         <v>258</v>
       </c>
-      <c r="H14" s="45" t="s">
+      <c r="H14" s="36" t="s">
         <v>222</v>
       </c>
-      <c r="K14" s="35"/>
+      <c r="K14" s="26"/>
     </row>
     <row r="15" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B15" s="44">
+      <c r="B15" s="35">
         <v>11</v>
       </c>
       <c r="C15" s="25" t="s">
@@ -74971,17 +77169,17 @@
       <c r="E15" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="F15" s="45"/>
-      <c r="G15" s="45" t="s">
+      <c r="F15" s="36"/>
+      <c r="G15" s="36" t="s">
         <v>263</v>
       </c>
-      <c r="H15" s="45" t="s">
+      <c r="H15" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="K15" s="35"/>
+      <c r="K15" s="26"/>
     </row>
     <row r="16" spans="2:11" s="11" customFormat="1" ht="130">
-      <c r="B16" s="44">
+      <c r="B16" s="35">
         <v>12</v>
       </c>
       <c r="C16" s="25" t="s">
@@ -74993,19 +77191,19 @@
       <c r="E16" s="25" t="s">
         <v>259</v>
       </c>
-      <c r="F16" s="45" t="s">
+      <c r="F16" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G16" s="45" t="s">
+      <c r="G16" s="36" t="s">
         <v>264</v>
       </c>
-      <c r="H16" s="45" t="s">
+      <c r="H16" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="K16" s="35"/>
+      <c r="K16" s="26"/>
     </row>
     <row r="17" spans="2:11" s="11" customFormat="1" ht="65">
-      <c r="B17" s="44">
+      <c r="B17" s="35">
         <v>13</v>
       </c>
       <c r="C17" s="25" t="s">
@@ -75017,19 +77215,19 @@
       <c r="E17" s="25" t="s">
         <v>204</v>
       </c>
-      <c r="F17" s="45" t="s">
+      <c r="F17" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G17" s="45" t="s">
+      <c r="G17" s="36" t="s">
         <v>265</v>
       </c>
-      <c r="H17" s="45" t="s">
+      <c r="H17" s="36" t="s">
         <v>225</v>
       </c>
-      <c r="K17" s="35"/>
+      <c r="K17" s="26"/>
     </row>
     <row r="18" spans="2:11" s="11" customFormat="1" ht="65">
-      <c r="B18" s="44">
+      <c r="B18" s="35">
         <v>14</v>
       </c>
       <c r="C18" s="25" t="s">
@@ -75041,19 +77239,19 @@
       <c r="E18" s="25" t="s">
         <v>260</v>
       </c>
-      <c r="F18" s="45" t="s">
+      <c r="F18" s="36" t="s">
         <v>164</v>
       </c>
-      <c r="G18" s="45" t="s">
+      <c r="G18" s="36" t="s">
         <v>266</v>
       </c>
-      <c r="H18" s="45" t="s">
+      <c r="H18" s="36" t="s">
         <v>226</v>
       </c>
-      <c r="K18" s="35"/>
+      <c r="K18" s="26"/>
     </row>
     <row r="19" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B19" s="44">
+      <c r="B19" s="35">
         <v>15</v>
       </c>
       <c r="C19" s="25" t="s">
@@ -75065,19 +77263,19 @@
       <c r="E19" s="25" t="s">
         <v>205</v>
       </c>
-      <c r="F19" s="45" t="s">
+      <c r="F19" s="36" t="s">
         <v>107</v>
       </c>
-      <c r="G19" s="45" t="s">
+      <c r="G19" s="36" t="s">
         <v>267</v>
       </c>
-      <c r="H19" s="45" t="s">
+      <c r="H19" s="36" t="s">
         <v>227</v>
       </c>
-      <c r="K19" s="35"/>
+      <c r="K19" s="26"/>
     </row>
     <row r="20" spans="2:11" s="11" customFormat="1" ht="65">
-      <c r="B20" s="44">
+      <c r="B20" s="35">
         <v>16</v>
       </c>
       <c r="C20" s="25" t="s">
@@ -75089,19 +77287,19 @@
       <c r="E20" s="25" t="s">
         <v>268</v>
       </c>
-      <c r="F20" s="45" t="s">
+      <c r="F20" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="G20" s="45" t="s">
+      <c r="G20" s="36" t="s">
         <v>274</v>
       </c>
-      <c r="H20" s="45" t="s">
+      <c r="H20" s="36" t="s">
         <v>228</v>
       </c>
-      <c r="K20" s="35"/>
+      <c r="K20" s="26"/>
     </row>
     <row r="21" spans="2:11" s="11" customFormat="1" ht="78">
-      <c r="B21" s="44">
+      <c r="B21" s="35">
         <v>17</v>
       </c>
       <c r="C21" s="25" t="s">
@@ -75113,19 +77311,19 @@
       <c r="E21" s="25" t="s">
         <v>206</v>
       </c>
-      <c r="F21" s="45" t="s">
+      <c r="F21" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="G21" s="45" t="s">
+      <c r="G21" s="36" t="s">
         <v>275</v>
       </c>
-      <c r="H21" s="45" t="s">
+      <c r="H21" s="36" t="s">
         <v>229</v>
       </c>
-      <c r="K21" s="35"/>
+      <c r="K21" s="26"/>
     </row>
     <row r="22" spans="2:11" s="11" customFormat="1" ht="65">
-      <c r="B22" s="44">
+      <c r="B22" s="35">
         <v>18</v>
       </c>
       <c r="C22" s="25" t="s">
@@ -75137,19 +77335,19 @@
       <c r="E22" s="25" t="s">
         <v>269</v>
       </c>
-      <c r="F22" s="45" t="s">
+      <c r="F22" s="36" t="s">
         <v>165</v>
       </c>
-      <c r="G22" s="45" t="s">
+      <c r="G22" s="36" t="s">
         <v>276</v>
       </c>
-      <c r="H22" s="45" t="s">
+      <c r="H22" s="36" t="s">
         <v>230</v>
       </c>
-      <c r="K22" s="35"/>
+      <c r="K22" s="26"/>
     </row>
     <row r="23" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B23" s="44">
+      <c r="B23" s="35">
         <v>19</v>
       </c>
       <c r="C23" s="25" t="s">
@@ -75161,17 +77359,17 @@
       <c r="E23" s="25" t="s">
         <v>124</v>
       </c>
-      <c r="F23" s="45"/>
-      <c r="G23" s="45" t="s">
+      <c r="F23" s="36"/>
+      <c r="G23" s="36" t="s">
         <v>277</v>
       </c>
-      <c r="H23" s="45" t="s">
+      <c r="H23" s="36" t="s">
         <v>231</v>
       </c>
-      <c r="K23" s="35"/>
+      <c r="K23" s="26"/>
     </row>
     <row r="24" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B24" s="44">
+      <c r="B24" s="35">
         <v>20</v>
       </c>
       <c r="C24" s="25" t="s">
@@ -75183,17 +77381,17 @@
       <c r="E24" s="25" t="s">
         <v>207</v>
       </c>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45" t="s">
+      <c r="F24" s="36"/>
+      <c r="G24" s="36" t="s">
         <v>278</v>
       </c>
-      <c r="H24" s="45" t="s">
+      <c r="H24" s="36" t="s">
         <v>232</v>
       </c>
-      <c r="K24" s="35"/>
+      <c r="K24" s="26"/>
     </row>
     <row r="25" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B25" s="44">
+      <c r="B25" s="35">
         <v>21</v>
       </c>
       <c r="C25" s="25" t="s">
@@ -75205,19 +77403,19 @@
       <c r="E25" s="25" t="s">
         <v>270</v>
       </c>
-      <c r="F25" s="45" t="s">
+      <c r="F25" s="36" t="s">
         <v>161</v>
       </c>
-      <c r="G25" s="45" t="s">
+      <c r="G25" s="36" t="s">
         <v>279</v>
       </c>
-      <c r="H25" s="45" t="s">
+      <c r="H25" s="36" t="s">
         <v>233</v>
       </c>
-      <c r="K25" s="35"/>
+      <c r="K25" s="26"/>
     </row>
     <row r="26" spans="2:11" s="11" customFormat="1" ht="65">
-      <c r="B26" s="44">
+      <c r="B26" s="35">
         <v>22</v>
       </c>
       <c r="C26" s="25" t="s">
@@ -75229,19 +77427,19 @@
       <c r="E26" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="F26" s="45" t="s">
+      <c r="F26" s="36" t="s">
         <v>163</v>
       </c>
-      <c r="G26" s="45" t="s">
+      <c r="G26" s="36" t="s">
         <v>280</v>
       </c>
-      <c r="H26" s="45" t="s">
+      <c r="H26" s="36" t="s">
         <v>234</v>
       </c>
-      <c r="K26" s="35"/>
+      <c r="K26" s="26"/>
     </row>
     <row r="27" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B27" s="44">
+      <c r="B27" s="35">
         <v>23</v>
       </c>
       <c r="C27" s="25" t="s">
@@ -75253,15 +77451,15 @@
       <c r="E27" s="25" t="s">
         <v>208</v>
       </c>
-      <c r="F27" s="45"/>
-      <c r="G27" s="45"/>
-      <c r="H27" s="45" t="s">
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36" t="s">
         <v>235</v>
       </c>
-      <c r="K27" s="35"/>
+      <c r="K27" s="26"/>
     </row>
     <row r="28" spans="2:11" s="11" customFormat="1" ht="46">
-      <c r="B28" s="44">
+      <c r="B28" s="35">
         <v>24</v>
       </c>
       <c r="C28" s="25" t="s">
@@ -75274,16 +77472,16 @@
         <v>209</v>
       </c>
       <c r="F28" s="22"/>
-      <c r="G28" s="45" t="s">
+      <c r="G28" s="36" t="s">
         <v>281</v>
       </c>
-      <c r="H28" s="45" t="s">
+      <c r="H28" s="36" t="s">
         <v>236</v>
       </c>
-      <c r="K28" s="35"/>
+      <c r="K28" s="26"/>
     </row>
     <row r="29" spans="2:11" s="11" customFormat="1" ht="69">
-      <c r="B29" s="44">
+      <c r="B29" s="35">
         <v>25</v>
       </c>
       <c r="C29" s="25" t="s">
@@ -75296,16 +77494,16 @@
         <v>272</v>
       </c>
       <c r="F29" s="22"/>
-      <c r="G29" s="45" t="s">
+      <c r="G29" s="36" t="s">
         <v>282</v>
       </c>
-      <c r="H29" s="45" t="s">
+      <c r="H29" s="36" t="s">
         <v>237</v>
       </c>
-      <c r="K29" s="35"/>
+      <c r="K29" s="26"/>
     </row>
     <row r="30" spans="2:11" s="11" customFormat="1" ht="13.5">
-      <c r="B30" s="44">
+      <c r="B30" s="35">
         <v>26</v>
       </c>
       <c r="C30" s="25" t="s">
@@ -75318,16 +77516,16 @@
         <v>273</v>
       </c>
       <c r="F30" s="22"/>
-      <c r="G30" s="45" t="s">
+      <c r="G30" s="36" t="s">
         <v>283</v>
       </c>
-      <c r="H30" s="45" t="s">
+      <c r="H30" s="36" t="s">
         <v>238</v>
       </c>
-      <c r="K30" s="35"/>
+      <c r="K30" s="26"/>
     </row>
     <row r="31" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B31" s="44">
+      <c r="B31" s="35">
         <v>27</v>
       </c>
       <c r="C31" s="25" t="s">
@@ -75339,17 +77537,17 @@
       <c r="E31" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45" t="s">
+      <c r="F31" s="36"/>
+      <c r="G31" s="36" t="s">
         <v>284</v>
       </c>
-      <c r="H31" s="45" t="s">
+      <c r="H31" s="36" t="s">
         <v>239</v>
       </c>
-      <c r="K31" s="35"/>
+      <c r="K31" s="26"/>
     </row>
     <row r="32" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B32" s="44">
+      <c r="B32" s="35">
         <v>28</v>
       </c>
       <c r="C32" s="25" t="s">
@@ -75361,17 +77559,17 @@
       <c r="E32" s="25" t="s">
         <v>285</v>
       </c>
-      <c r="F32" s="45"/>
-      <c r="G32" s="45" t="s">
+      <c r="F32" s="36"/>
+      <c r="G32" s="36" t="s">
         <v>288</v>
       </c>
-      <c r="H32" s="45" t="s">
+      <c r="H32" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="K32" s="35"/>
+      <c r="K32" s="26"/>
     </row>
     <row r="33" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B33" s="44">
+      <c r="B33" s="35">
         <v>29</v>
       </c>
       <c r="C33" s="25" t="s">
@@ -75383,17 +77581,17 @@
       <c r="E33" s="25" t="s">
         <v>210</v>
       </c>
-      <c r="F33" s="45"/>
-      <c r="G33" s="45" t="s">
+      <c r="F33" s="36"/>
+      <c r="G33" s="36" t="s">
         <v>289</v>
       </c>
-      <c r="H33" s="45" t="s">
+      <c r="H33" s="36" t="s">
         <v>241</v>
       </c>
-      <c r="K33" s="35"/>
+      <c r="K33" s="26"/>
     </row>
     <row r="34" spans="2:11" s="11" customFormat="1" ht="104">
-      <c r="B34" s="44">
+      <c r="B34" s="35">
         <v>30</v>
       </c>
       <c r="C34" s="25" t="s">
@@ -75405,19 +77603,19 @@
       <c r="E34" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="F34" s="45" t="s">
+      <c r="F34" s="36" t="s">
         <v>162</v>
       </c>
-      <c r="G34" s="45" t="s">
+      <c r="G34" s="36" t="s">
         <v>290</v>
       </c>
-      <c r="H34" s="45" t="s">
+      <c r="H34" s="36" t="s">
         <v>242</v>
       </c>
-      <c r="K34" s="35"/>
+      <c r="K34" s="26"/>
     </row>
     <row r="35" spans="2:11" s="11" customFormat="1" ht="52">
-      <c r="B35" s="44">
+      <c r="B35" s="35">
         <v>31</v>
       </c>
       <c r="C35" s="25" t="s">
@@ -75429,17 +77627,17 @@
       <c r="E35" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="F35" s="45"/>
-      <c r="G35" s="45" t="s">
+      <c r="F35" s="36"/>
+      <c r="G35" s="36" t="s">
         <v>291</v>
       </c>
-      <c r="H35" s="45" t="s">
+      <c r="H35" s="36" t="s">
         <v>243</v>
       </c>
-      <c r="K35" s="35"/>
+      <c r="K35" s="26"/>
     </row>
     <row r="36" spans="2:11" s="11" customFormat="1" ht="39">
-      <c r="B36" s="44">
+      <c r="B36" s="35">
         <v>32</v>
       </c>
       <c r="C36" s="25" t="s">
@@ -75451,19 +77649,19 @@
       <c r="E36" s="25" t="s">
         <v>286</v>
       </c>
-      <c r="F36" s="45" t="s">
+      <c r="F36" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="G36" s="45" t="s">
+      <c r="G36" s="36" t="s">
         <v>292</v>
       </c>
-      <c r="H36" s="45" t="s">
+      <c r="H36" s="36" t="s">
         <v>244</v>
       </c>
-      <c r="K36" s="35"/>
+      <c r="K36" s="26"/>
     </row>
     <row r="37" spans="2:11" ht="65">
-      <c r="B37" s="44">
+      <c r="B37" s="35">
         <v>33</v>
       </c>
       <c r="C37" s="25" t="s">
@@ -75475,18 +77673,18 @@
       <c r="E37" s="25" t="s">
         <v>287</v>
       </c>
-      <c r="F37" s="45" t="s">
+      <c r="F37" s="36" t="s">
         <v>42</v>
       </c>
       <c r="G37" s="22" t="s">
         <v>293</v>
       </c>
-      <c r="H37" s="45" t="s">
+      <c r="H37" s="36" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="38" spans="2:11" ht="79.5" customHeight="1">
-      <c r="B38" s="44">
+      <c r="B38" s="35">
         <v>34</v>
       </c>
       <c r="C38" s="25" t="s">
@@ -75498,14 +77696,35 @@
       <c r="E38" s="25" t="s">
         <v>211</v>
       </c>
-      <c r="F38" s="45" t="s">
+      <c r="F38" s="36" t="s">
         <v>52</v>
       </c>
       <c r="G38" s="22" t="s">
         <v>294</v>
       </c>
-      <c r="H38" s="45" t="s">
+      <c r="H38" s="36" t="s">
         <v>246</v>
+      </c>
+    </row>
+    <row r="39" spans="2:11" ht="130">
+      <c r="B39" s="35">
+        <v>35</v>
+      </c>
+      <c r="C39" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="D39" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="E39" s="25" t="s">
+        <v>297</v>
+      </c>
+      <c r="F39" s="36"/>
+      <c r="G39" s="37" t="s">
+        <v>298</v>
+      </c>
+      <c r="H39" s="36" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>
@@ -75515,7 +77734,7 @@
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C38">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C39">
       <formula1>$K$4:$K$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update scripts and data files: 36_프로젝트종결보고
</commit_message>
<xml_diff>
--- a/data/자동화태스크.xlsx
+++ b/data/자동화태스크.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWork\MySite\stComm\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWork\MySite\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="303">
   <si>
     <r>
       <rPr>
@@ -75120,6 +75120,1558 @@
   </si>
   <si>
     <t>35_프로젝트계획서최신화이력관리.html</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>IHANS_PRO_2026_036</t>
+  </si>
+  <si>
+    <t>36_36_프로젝트종결보고.html</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>연간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수십</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>건에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이르는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>경우에는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보고서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동화가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>효율적이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>대비</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>실적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>비교를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기본으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고서는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매칭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>구조로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">설계
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트계획서로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>부터</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>인용해서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사용한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>템플릿에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>실제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>현황은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>입력한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>. (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>향후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>산출물에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>인용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>예정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고서는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>단계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>승인을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>거치도록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>첫째</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수행팀에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검토</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>, (1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>차</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>승인을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행하며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">,  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>둘째</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>책임자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>스폰서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>또는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>그</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이상의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보직자가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보고서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>전체에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>대한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>차</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최종</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>승인을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -76865,7 +78417,7 @@
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K39"/>
+  <dimension ref="B2:K40"/>
   <sheetFormatPr defaultRowHeight="11.5"/>
   <cols>
     <col min="1" max="1" width="2.58203125" style="2" customWidth="1"/>
@@ -77727,6 +79279,27 @@
         <v>295</v>
       </c>
     </row>
+    <row r="40" spans="2:11" ht="104">
+      <c r="B40" s="35">
+        <v>36</v>
+      </c>
+      <c r="C40" s="25" t="s">
+        <v>184</v>
+      </c>
+      <c r="D40" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="F40" s="36"/>
+      <c r="G40" s="37" t="s">
+        <v>300</v>
+      </c>
+      <c r="H40" s="36" t="s">
+        <v>299</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="B5:F38">
     <sortCondition ref="C5:C38"/>
@@ -77734,7 +79307,7 @@
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C39">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C40">
       <formula1>$K$4:$K$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Update scripts and data files: 36_프로젝트종결보고 관련  수정
</commit_message>
<xml_diff>
--- a/data/자동화태스크.xlsx
+++ b/data/자동화태스크.xlsx
@@ -75126,410 +75126,1499 @@
     <t>IHANS_PRO_2026_036</t>
   </si>
   <si>
-    <t>36_36_프로젝트종결보고.html</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>연간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수십</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>건에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이르는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>경우에는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보고서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동화가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>효율적이다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>대비</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>실적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>비교를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기본으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획서와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고서는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매칭</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>구조로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">설계
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>계획은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트계획서로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>부터</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>인용해서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사용한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">.
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>템플릿에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>실제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>현황은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>입력한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>. (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>향후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>산출물에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>인용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>예정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결보고서는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>단계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>승인을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>거치도록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. 
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>첫째</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수행팀에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검토</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>, (1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>차</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>승인을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행하며</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">,  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>둘째</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프로젝트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>책임자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>스폰서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>또는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>그</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이상의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보직자가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>종결</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>보고서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>전체에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>대한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>차</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최종</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>승인을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>한다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.</t>
+    </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>▷</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>연간</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>수행</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>프로젝트가</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>수십</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>건에</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>이르는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>경우에는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>보고서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>자동화가</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>효율적이다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>▷</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결보고는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>계획</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>대비</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>실적</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>비교를</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>기본으로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">.
-    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
+      <t xml:space="preserve">• </t>
     </r>
     <r>
       <rPr>
@@ -75558,657 +76647,7 @@
         <family val="3"/>
         <charset val="129"/>
       </rPr>
-      <t>계획서와</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결보고서는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>매칭</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>구조로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">설계
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>계획은</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>프로젝트계획서로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>부터</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>자동</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>인용해서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>사용한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">.
-    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>템플릿에서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>실제</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>현황은</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>수기</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>입력한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>. (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>향후</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>산출물에서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>자동</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>인용</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>자동화</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>예정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">)
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>▷</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결보고서는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> 2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>단계</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>승인을</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>거치도록</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">. 
-    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>첫째</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>프로젝트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>수행팀에서</t>
+      <t>종결보고서</t>
     </r>
     <r>
       <rPr>
@@ -76228,450 +76667,11 @@
         <charset val="129"/>
       </rPr>
       <t>작성</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>검토</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>, (1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>차</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>승인을</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>진행하며</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">,  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>둘째</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>프로젝트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>책임자</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>스폰서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>또는</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>그</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>이상의</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>보직자가</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>보고서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>전체에</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>대한</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>차</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>최종</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>승인을</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>한다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>.</t>
     </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">• </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>프로젝트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>종결보고서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>작성</t>
-    </r>
+    <t>36_프로젝트종결보고.html</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -79287,14 +79287,14 @@
         <v>184</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E40" s="25" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F40" s="36"/>
       <c r="G40" s="37" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="H40" s="36" t="s">
         <v>299</v>

</xml_diff>

<commit_message>
Add two tasks, 037_SW로직설계, 038_SW테스트케이스설계
</commit_message>
<xml_diff>
--- a/data/자동화태스크.xlsx
+++ b/data/자동화태스크.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWork\MySite\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyWork\MySite\stComm\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -15,7 +15,7 @@
     <sheet name="SW프로젝트 관리자동화" sheetId="1" r:id="rId1"/>
     <sheet name="SWPJT_Web" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="152511" iterateDelta="1E-4"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="303">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="311">
   <si>
     <r>
       <rPr>
@@ -76674,12 +76674,2856 @@
     <t>36_프로젝트종결보고.html</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
+  <si>
+    <t>IHANS_PRO_2026_037</t>
+  </si>
+  <si>
+    <t>IHANS_PRO_2026_038</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="바탕"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(+LLM)</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>37_SW로직설계.html</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>38_SW테스트케이스설계.html</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">• SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(+LLM)</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>레거시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>코드와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계요구조건을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기반으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>소프트웨어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">수행
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최초</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>개발</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계요구조건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (LLM) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프롬프트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>구조화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (LLM) SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">(draft) + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>플로우차트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> + Ascet/Simulink </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가이드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">(c code </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>방식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>파생개발</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>또는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>유지보수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계요구조건</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (LLM) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>프롬프트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>구조화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>레거시</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>코드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (LLM) SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">(draft) + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>플로우차트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> + Ascet/Simulink </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가이드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">(c code </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>방식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">
+▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계요구조건은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 1) PDF, 2) txt, 3) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>엑셀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>시트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>셀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>참조</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(SR</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>엑셀</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>시트로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>변환한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>경우</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">), 4) inputbox </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>입력</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>업로딩
+▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> 1) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>성능</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자원</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최적화형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 2) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>가독성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>유지보수형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 3) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>안전성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>예외처리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>강화형</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>옵션으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>. 1)~3)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>택일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>또는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>복수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>선택으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최종</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계
+▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(draft)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>과정에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검증</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>업무를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>산정하기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>위해</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>도출</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>향후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계와</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>비교에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>활용</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> MBD(Ascet/Simulink </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>외</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> auto generated </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>또는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매뉴얼로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작성한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>코드를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기반으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> AST </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>파서를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이용하여</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>코드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>단위로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">작성
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>펌웨어</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>탑재용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최종</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>코드로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검증을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>위한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>최소한의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">제안
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>함수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>운용은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> SW</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>템플릿과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>공용이지만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>결과는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>별도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>파일에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>기록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>V-Cycle</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>상의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검증</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>산출물로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>활용
+▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> SW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>로직</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>설계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>과정에서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>도출한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(draft)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>상호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>비교를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>통해</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>테스트케이스의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>적정성을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>점검</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="19">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76807,6 +79651,13 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="바탕"/>
+      <family val="1"/>
+      <charset val="129"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF303030"/>
       <name val="바탕"/>
       <family val="1"/>
       <charset val="129"/>
@@ -78417,7 +81268,7 @@
   <sheetPr codeName="Sheet4">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:K40"/>
+  <dimension ref="B2:K42"/>
   <sheetFormatPr defaultRowHeight="11.5"/>
   <cols>
     <col min="1" max="1" width="2.58203125" style="2" customWidth="1"/>
@@ -79300,6 +82151,52 @@
         <v>299</v>
       </c>
     </row>
+    <row r="41" spans="2:11" ht="117">
+      <c r="B41" s="35">
+        <v>37</v>
+      </c>
+      <c r="C41" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="D41" s="25" t="s">
+        <v>305</v>
+      </c>
+      <c r="E41" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="F41" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="G41" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="H41" s="36" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="42" spans="2:11" ht="91">
+      <c r="B42" s="35">
+        <v>38</v>
+      </c>
+      <c r="C42" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="D42" s="25" t="s">
+        <v>308</v>
+      </c>
+      <c r="E42" s="25" t="s">
+        <v>310</v>
+      </c>
+      <c r="F42" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="G42" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="H42" s="36" t="s">
+        <v>304</v>
+      </c>
+    </row>
   </sheetData>
   <sortState ref="B5:F38">
     <sortCondition ref="C5:C38"/>
@@ -79307,7 +82204,7 @@
   </sortState>
   <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C40">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C5:C42">
       <formula1>$K$4:$K$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
change diagram and add 14-2 cve monthly monitoring
</commit_message>
<xml_diff>
--- a/data/자동화태스크.xlsx
+++ b/data/자동화태스크.xlsx
@@ -64285,907 +64285,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>▷</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>사이버보안</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>개발</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>후</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>활동으로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>취약점</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>모니터링</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>업무를</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">자동화
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> VBA-Python </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>브릿지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>방식으로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">개발
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>데일리</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>검색</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>및</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>주기적</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>검색</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>월간</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>방식</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>모두</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">가능
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>ㄴ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>데일리</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>검색은</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>윈도우</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>태스크</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>스케줄러를</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>이용하여</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>매일</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>정해진</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>시각에</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>자동수행</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">
-▷</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>사이버보안의</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>경우</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">, CRA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>규제</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>강화로</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> SBOM </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>중요성</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>부각</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>→</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> SBOM </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>내</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>중요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>요소인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>오픈소스</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>모니터링에도</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF303030"/>
-        <rFont val="나눔고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t>적용</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <r>
       <t>2-1_</t>
     </r>
     <r>
@@ -65372,31 +64471,6 @@
         <charset val="129"/>
       </rPr>
       <t>자동화</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>.html</t>
-    </r>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>14_CVE</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="바탕"/>
-        <family val="1"/>
-        <charset val="129"/>
-      </rPr>
-      <t>취약점모니터링</t>
     </r>
     <r>
       <rPr>
@@ -81388,6 +80462,1839 @@
         <charset val="129"/>
       </rPr>
       <t>보완</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>14_CVE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="바탕"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t>취약점모니터링</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.html,
+14-2_CVE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="바탕"/>
+        <family val="1"/>
+        <charset val="129"/>
+      </rPr>
+      <t>취약점월간모니터링</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>.html</t>
+    </r>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사이버보안</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>개발</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>활동으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>취약점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모니터링</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>업무를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">자동화
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> VBA-Python </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>브릿지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>방식으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">개발
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>데일리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검색</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>및</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>주기적</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검색</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>월간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>방식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모두</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">가능
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">        - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>데일리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>월간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모두</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>파이썬</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>스크립트만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>실행하면</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>분석을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>위한</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> CVE </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>데이터가</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수집</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매뉴얼</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>작업</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>없음</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>데일리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>검색은</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>윈도우</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>태스크</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>스케줄러를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이용하여</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정해진</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>시각에</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동수행
+▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>취약점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수집</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>후에는</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>매뉴얼로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>분석</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수행</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>중간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>점검을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>목적으로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>완전</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>자동화를</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>지양함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>▷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>사이버보안의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>경우</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, CRA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>규제</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>강화로</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> SBOM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>중요성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>부각</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>→</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> SBOM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>내</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>중요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>요소인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>오픈소스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모니터링에도</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">적용
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>데일리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>월간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>방식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>모두</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>적용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t xml:space="preserve">가능
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>ㄴ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>수집</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>정보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>중간</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>점검</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>이후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>오픈소스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>분석을</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF303030"/>
+        <rFont val="나눔고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+      </rPr>
+      <t>진행</t>
     </r>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -83204,7 +84111,7 @@
         <v>184</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>198</v>
@@ -83238,7 +84145,7 @@
         <v>37</v>
       </c>
       <c r="G6" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H6" s="36" t="s">
         <v>214</v>
@@ -83264,7 +84171,7 @@
         <v>37</v>
       </c>
       <c r="G7" s="36" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="H7" s="36" t="s">
         <v>215</v>
@@ -83374,7 +84281,7 @@
         <v>188</v>
       </c>
       <c r="D12" s="25" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E12" s="25" t="s">
         <v>251</v>
@@ -83447,7 +84354,7 @@
       </c>
       <c r="F15" s="36"/>
       <c r="G15" s="36" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="H15" s="36" t="s">
         <v>223</v>
@@ -83471,7 +84378,7 @@
         <v>37</v>
       </c>
       <c r="G16" s="36" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H16" s="36" t="s">
         <v>224</v>
@@ -83495,14 +84402,14 @@
         <v>37</v>
       </c>
       <c r="G17" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="H17" s="36" t="s">
         <v>225</v>
       </c>
       <c r="K17" s="26"/>
     </row>
-    <row r="18" spans="2:11" s="11" customFormat="1" ht="65">
+    <row r="18" spans="2:11" s="11" customFormat="1" ht="127.5" customHeight="1">
       <c r="B18" s="35">
         <v>14</v>
       </c>
@@ -83513,13 +84420,13 @@
         <v>98</v>
       </c>
       <c r="E18" s="25" t="s">
-        <v>260</v>
+        <v>315</v>
       </c>
       <c r="F18" s="36" t="s">
         <v>164</v>
       </c>
       <c r="G18" s="36" t="s">
-        <v>266</v>
+        <v>314</v>
       </c>
       <c r="H18" s="36" t="s">
         <v>226</v>
@@ -83543,7 +84450,7 @@
         <v>107</v>
       </c>
       <c r="G19" s="36" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H19" s="36" t="s">
         <v>227</v>
@@ -83561,13 +84468,13 @@
         <v>169</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="F20" s="36" t="s">
         <v>47</v>
       </c>
       <c r="G20" s="36" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H20" s="36" t="s">
         <v>228</v>
@@ -83591,7 +84498,7 @@
         <v>121</v>
       </c>
       <c r="G21" s="36" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H21" s="36" t="s">
         <v>229</v>
@@ -83609,13 +84516,13 @@
         <v>112</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F22" s="36" t="s">
         <v>165</v>
       </c>
       <c r="G22" s="36" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H22" s="36" t="s">
         <v>230</v>
@@ -83637,7 +84544,7 @@
       </c>
       <c r="F23" s="36"/>
       <c r="G23" s="36" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H23" s="36" t="s">
         <v>231</v>
@@ -83659,7 +84566,7 @@
       </c>
       <c r="F24" s="36"/>
       <c r="G24" s="36" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H24" s="36" t="s">
         <v>232</v>
@@ -83677,13 +84584,13 @@
         <v>17</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F25" s="36" t="s">
         <v>161</v>
       </c>
       <c r="G25" s="36" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="H25" s="36" t="s">
         <v>233</v>
@@ -83707,7 +84614,7 @@
         <v>163</v>
       </c>
       <c r="G26" s="36" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="H26" s="36" t="s">
         <v>234</v>
@@ -83749,7 +84656,7 @@
       </c>
       <c r="F28" s="22"/>
       <c r="G28" s="36" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="H28" s="36" t="s">
         <v>236</v>
@@ -83767,11 +84674,11 @@
         <v>181</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F29" s="22"/>
       <c r="G29" s="36" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H29" s="36" t="s">
         <v>237</v>
@@ -83789,11 +84696,11 @@
         <v>180</v>
       </c>
       <c r="E30" s="24" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F30" s="22"/>
       <c r="G30" s="36" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H30" s="36" t="s">
         <v>238</v>
@@ -83815,7 +84722,7 @@
       </c>
       <c r="F31" s="36"/>
       <c r="G31" s="36" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H31" s="36" t="s">
         <v>239</v>
@@ -83833,11 +84740,11 @@
         <v>25</v>
       </c>
       <c r="E32" s="25" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F32" s="36"/>
       <c r="G32" s="36" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="H32" s="36" t="s">
         <v>240</v>
@@ -83859,7 +84766,7 @@
       </c>
       <c r="F33" s="36"/>
       <c r="G33" s="36" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H33" s="36" t="s">
         <v>241</v>
@@ -83883,7 +84790,7 @@
         <v>162</v>
       </c>
       <c r="G34" s="36" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="H34" s="36" t="s">
         <v>242</v>
@@ -83905,7 +84812,7 @@
       </c>
       <c r="F35" s="36"/>
       <c r="G35" s="36" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H35" s="36" t="s">
         <v>243</v>
@@ -83923,13 +84830,13 @@
         <v>167</v>
       </c>
       <c r="E36" s="25" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F36" s="36" t="s">
         <v>37</v>
       </c>
       <c r="G36" s="36" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="H36" s="36" t="s">
         <v>244</v>
@@ -83947,13 +84854,13 @@
         <v>168</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="F37" s="36" t="s">
         <v>42</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="H37" s="36" t="s">
         <v>245</v>
@@ -83976,7 +84883,7 @@
         <v>52</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="H38" s="36" t="s">
         <v>246</v>
@@ -83990,17 +84897,17 @@
         <v>184</v>
       </c>
       <c r="D39" s="25" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="F39" s="36"/>
       <c r="G39" s="37" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="H39" s="36" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="40" spans="2:11" ht="104">
@@ -84011,17 +84918,17 @@
         <v>184</v>
       </c>
       <c r="D40" s="25" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E40" s="25" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="F40" s="36"/>
       <c r="G40" s="37" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="H40" s="36" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="41" spans="2:11" ht="117">
@@ -84032,19 +84939,19 @@
         <v>188</v>
       </c>
       <c r="D41" s="25" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E41" s="25" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="F41" s="36" t="s">
         <v>37</v>
       </c>
       <c r="G41" s="37" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="H41" s="36" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
     </row>
     <row r="42" spans="2:11" ht="91">
@@ -84055,19 +84962,19 @@
         <v>188</v>
       </c>
       <c r="D42" s="25" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="E42" s="25" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="F42" s="36" t="s">
         <v>37</v>
       </c>
       <c r="G42" s="37" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="H42" s="36" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="43" spans="2:11" ht="117">
@@ -84078,19 +84985,19 @@
         <v>188</v>
       </c>
       <c r="D43" s="25" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="F43" s="36" t="s">
         <v>37</v>
       </c>
       <c r="G43" s="37" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="H43" s="36" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>